<commit_message>
OLED link added in BOMs #49
</commit_message>
<xml_diff>
--- a/Design Files/Baseboard-v3.0/BOM/JLCPCB-BOM-Baseboard-v3.0-Core.xlsx
+++ b/Design Files/Baseboard-v3.0/BOM/JLCPCB-BOM-Baseboard-v3.0-Core.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="470">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="577" uniqueCount="474">
   <si>
     <t>Comment</t>
   </si>
@@ -1421,6 +1421,18 @@
   </si>
   <si>
     <t>C99009</t>
+  </si>
+  <si>
+    <t>OLED</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Custom</t>
+  </si>
+  <si>
+    <t>C2890594</t>
   </si>
 </sst>
 </file>
@@ -1563,7 +1575,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1585,9 +1597,6 @@
     <xf borderId="6" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="5" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
     <xf quotePrefix="1" borderId="3" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
@@ -1599,6 +1608,12 @@
     </xf>
     <xf quotePrefix="1" borderId="7" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
@@ -3053,7 +3068,7 @@
       <c r="A89" s="5" t="s">
         <v>291</v>
       </c>
-      <c r="B89" s="7" t="s">
+      <c r="B89" s="5" t="s">
         <v>292</v>
       </c>
       <c r="C89" s="6" t="s">
@@ -3095,7 +3110,7 @@
       <c r="A92" s="3" t="s">
         <v>299</v>
       </c>
-      <c r="B92" s="8" t="s">
+      <c r="B92" s="7" t="s">
         <v>300</v>
       </c>
       <c r="C92" s="4" t="s">
@@ -3302,16 +3317,16 @@
       </c>
     </row>
     <row r="107" ht="15.75" customHeight="1">
-      <c r="A107" s="9" t="s">
+      <c r="A107" s="8" t="s">
         <v>334</v>
       </c>
-      <c r="B107" s="9" t="s">
+      <c r="B107" s="8" t="s">
         <v>346</v>
       </c>
-      <c r="C107" s="10" t="s">
+      <c r="C107" s="9" t="s">
         <v>273</v>
       </c>
-      <c r="D107" s="9" t="s">
+      <c r="D107" s="8" t="s">
         <v>301</v>
       </c>
     </row>
@@ -3470,44 +3485,44 @@
       </c>
     </row>
     <row r="119" ht="15.75" customHeight="1">
-      <c r="A119" s="9" t="s">
+      <c r="A119" s="8" t="s">
         <v>375</v>
       </c>
-      <c r="B119" s="9" t="s">
+      <c r="B119" s="8" t="s">
         <v>376</v>
       </c>
-      <c r="C119" s="10" t="s">
+      <c r="C119" s="9" t="s">
         <v>273</v>
       </c>
-      <c r="D119" s="9" t="s">
+      <c r="D119" s="8" t="s">
         <v>377</v>
       </c>
     </row>
     <row r="120" ht="15.75" customHeight="1">
-      <c r="A120" s="9" t="s">
+      <c r="A120" s="8" t="s">
         <v>378</v>
       </c>
-      <c r="B120" s="9" t="s">
+      <c r="B120" s="8" t="s">
         <v>379</v>
       </c>
-      <c r="C120" s="10" t="s">
+      <c r="C120" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="D120" s="9" t="s">
+      <c r="D120" s="8" t="s">
         <v>380</v>
       </c>
     </row>
     <row r="121" ht="15.75" customHeight="1">
-      <c r="A121" s="9" t="s">
+      <c r="A121" s="8" t="s">
         <v>381</v>
       </c>
-      <c r="B121" s="9" t="s">
+      <c r="B121" s="8" t="s">
         <v>382</v>
       </c>
-      <c r="C121" s="10" t="s">
+      <c r="C121" s="9" t="s">
         <v>273</v>
       </c>
-      <c r="D121" s="9" t="s">
+      <c r="D121" s="8" t="s">
         <v>383</v>
       </c>
     </row>
@@ -3515,7 +3530,7 @@
       <c r="A122" s="5" t="s">
         <v>384</v>
       </c>
-      <c r="B122" s="7" t="s">
+      <c r="B122" s="5" t="s">
         <v>385</v>
       </c>
       <c r="C122" s="6" t="s">
@@ -3764,16 +3779,16 @@
       </c>
     </row>
     <row r="140" ht="15.75" customHeight="1">
-      <c r="A140" s="11" t="s">
+      <c r="A140" s="10" t="s">
         <v>450</v>
       </c>
-      <c r="B140" s="9" t="s">
+      <c r="B140" s="8" t="s">
         <v>451</v>
       </c>
-      <c r="C140" s="10" t="s">
+      <c r="C140" s="9" t="s">
         <v>452</v>
       </c>
-      <c r="D140" s="9" t="s">
+      <c r="D140" s="8" t="s">
         <v>453</v>
       </c>
     </row>
@@ -3834,604 +3849,615 @@
       </c>
     </row>
     <row r="145" ht="15.75" customHeight="1">
-      <c r="A145" s="12"/>
+      <c r="A145" s="11" t="s">
+        <v>470</v>
+      </c>
+      <c r="B145" s="11" t="s">
+        <v>471</v>
+      </c>
+      <c r="C145" s="12" t="s">
+        <v>472</v>
+      </c>
+      <c r="D145" s="11" t="s">
+        <v>473</v>
+      </c>
     </row>
     <row r="146" ht="15.75" customHeight="1">
-      <c r="A146" s="12"/>
+      <c r="A146" s="13"/>
     </row>
     <row r="147" ht="15.75" customHeight="1">
-      <c r="A147" s="12"/>
+      <c r="A147" s="13"/>
     </row>
     <row r="148" ht="15.75" customHeight="1">
-      <c r="A148" s="12"/>
+      <c r="A148" s="13"/>
     </row>
     <row r="149" ht="15.75" customHeight="1">
-      <c r="A149" s="12"/>
+      <c r="A149" s="13"/>
     </row>
     <row r="150" ht="15.75" customHeight="1">
-      <c r="A150" s="12"/>
+      <c r="A150" s="13"/>
     </row>
     <row r="151" ht="15.75" customHeight="1">
-      <c r="A151" s="12"/>
+      <c r="A151" s="13"/>
     </row>
     <row r="152" ht="15.75" customHeight="1">
-      <c r="A152" s="12"/>
+      <c r="A152" s="13"/>
     </row>
     <row r="153" ht="15.75" customHeight="1">
-      <c r="A153" s="12"/>
+      <c r="A153" s="13"/>
     </row>
     <row r="154" ht="15.75" customHeight="1">
-      <c r="A154" s="12"/>
+      <c r="A154" s="13"/>
     </row>
     <row r="155" ht="15.75" customHeight="1">
-      <c r="A155" s="12"/>
+      <c r="A155" s="13"/>
     </row>
     <row r="156" ht="15.75" customHeight="1">
-      <c r="A156" s="12"/>
+      <c r="A156" s="13"/>
     </row>
     <row r="157" ht="15.75" customHeight="1">
-      <c r="A157" s="12"/>
+      <c r="A157" s="13"/>
     </row>
     <row r="158" ht="15.75" customHeight="1">
-      <c r="A158" s="12"/>
+      <c r="A158" s="13"/>
     </row>
     <row r="159" ht="15.75" customHeight="1">
-      <c r="A159" s="12"/>
+      <c r="A159" s="13"/>
     </row>
     <row r="160" ht="15.75" customHeight="1">
-      <c r="A160" s="12"/>
+      <c r="A160" s="13"/>
     </row>
     <row r="161" ht="15.75" customHeight="1">
-      <c r="A161" s="12"/>
+      <c r="A161" s="13"/>
     </row>
     <row r="162" ht="15.75" customHeight="1">
-      <c r="A162" s="12"/>
+      <c r="A162" s="13"/>
     </row>
     <row r="163" ht="15.75" customHeight="1">
-      <c r="A163" s="12"/>
+      <c r="A163" s="13"/>
     </row>
     <row r="164" ht="15.75" customHeight="1">
-      <c r="A164" s="12"/>
+      <c r="A164" s="13"/>
     </row>
     <row r="165" ht="15.75" customHeight="1">
-      <c r="A165" s="12"/>
+      <c r="A165" s="13"/>
     </row>
     <row r="166" ht="15.75" customHeight="1">
-      <c r="A166" s="12"/>
+      <c r="A166" s="13"/>
     </row>
     <row r="167" ht="15.75" customHeight="1">
-      <c r="A167" s="12"/>
+      <c r="A167" s="13"/>
     </row>
     <row r="168" ht="15.75" customHeight="1">
-      <c r="A168" s="12"/>
+      <c r="A168" s="13"/>
     </row>
     <row r="169" ht="15.75" customHeight="1">
-      <c r="A169" s="12"/>
+      <c r="A169" s="13"/>
     </row>
     <row r="170" ht="15.75" customHeight="1">
-      <c r="A170" s="12"/>
+      <c r="A170" s="13"/>
     </row>
     <row r="171" ht="15.75" customHeight="1">
-      <c r="A171" s="12"/>
+      <c r="A171" s="13"/>
     </row>
     <row r="172" ht="15.75" customHeight="1">
-      <c r="A172" s="12"/>
+      <c r="A172" s="13"/>
     </row>
     <row r="173" ht="15.75" customHeight="1">
-      <c r="A173" s="12"/>
+      <c r="A173" s="13"/>
     </row>
     <row r="174" ht="15.75" customHeight="1">
-      <c r="A174" s="12"/>
+      <c r="A174" s="13"/>
     </row>
     <row r="175" ht="15.75" customHeight="1">
-      <c r="A175" s="12"/>
+      <c r="A175" s="13"/>
     </row>
     <row r="176" ht="15.75" customHeight="1">
-      <c r="A176" s="12"/>
+      <c r="A176" s="13"/>
     </row>
     <row r="177" ht="15.75" customHeight="1">
-      <c r="A177" s="12"/>
+      <c r="A177" s="13"/>
     </row>
     <row r="178" ht="15.75" customHeight="1">
-      <c r="A178" s="12"/>
+      <c r="A178" s="13"/>
     </row>
     <row r="179" ht="15.75" customHeight="1">
-      <c r="A179" s="12"/>
+      <c r="A179" s="13"/>
     </row>
     <row r="180" ht="15.75" customHeight="1">
-      <c r="A180" s="12"/>
+      <c r="A180" s="13"/>
     </row>
     <row r="181" ht="15.75" customHeight="1">
-      <c r="A181" s="12"/>
+      <c r="A181" s="13"/>
     </row>
     <row r="182" ht="15.75" customHeight="1">
-      <c r="A182" s="12"/>
+      <c r="A182" s="13"/>
     </row>
     <row r="183" ht="15.75" customHeight="1">
-      <c r="A183" s="12"/>
+      <c r="A183" s="13"/>
     </row>
     <row r="184" ht="15.75" customHeight="1">
-      <c r="A184" s="12"/>
+      <c r="A184" s="13"/>
     </row>
     <row r="185" ht="15.75" customHeight="1">
-      <c r="A185" s="12"/>
+      <c r="A185" s="13"/>
     </row>
     <row r="186" ht="15.75" customHeight="1">
-      <c r="A186" s="12"/>
+      <c r="A186" s="13"/>
     </row>
     <row r="187" ht="15.75" customHeight="1">
-      <c r="A187" s="12"/>
+      <c r="A187" s="13"/>
     </row>
     <row r="188" ht="15.75" customHeight="1">
-      <c r="A188" s="12"/>
+      <c r="A188" s="13"/>
     </row>
     <row r="189" ht="15.75" customHeight="1">
-      <c r="A189" s="12"/>
+      <c r="A189" s="13"/>
     </row>
     <row r="190" ht="15.75" customHeight="1">
-      <c r="A190" s="12"/>
+      <c r="A190" s="13"/>
     </row>
     <row r="191" ht="15.75" customHeight="1">
-      <c r="A191" s="12"/>
+      <c r="A191" s="13"/>
     </row>
     <row r="192" ht="15.75" customHeight="1">
-      <c r="A192" s="12"/>
+      <c r="A192" s="13"/>
     </row>
     <row r="193" ht="15.75" customHeight="1">
-      <c r="A193" s="12"/>
+      <c r="A193" s="13"/>
     </row>
     <row r="194" ht="15.75" customHeight="1">
-      <c r="A194" s="12"/>
+      <c r="A194" s="13"/>
     </row>
     <row r="195" ht="15.75" customHeight="1">
-      <c r="A195" s="12"/>
+      <c r="A195" s="13"/>
     </row>
     <row r="196" ht="15.75" customHeight="1">
-      <c r="A196" s="12"/>
+      <c r="A196" s="13"/>
     </row>
     <row r="197" ht="15.75" customHeight="1">
-      <c r="A197" s="12"/>
+      <c r="A197" s="13"/>
     </row>
     <row r="198" ht="15.75" customHeight="1">
-      <c r="A198" s="12"/>
+      <c r="A198" s="13"/>
     </row>
     <row r="199" ht="15.75" customHeight="1">
-      <c r="A199" s="12"/>
+      <c r="A199" s="13"/>
     </row>
     <row r="200" ht="15.75" customHeight="1">
-      <c r="A200" s="12"/>
+      <c r="A200" s="13"/>
     </row>
     <row r="201" ht="15.75" customHeight="1">
-      <c r="A201" s="12"/>
+      <c r="A201" s="13"/>
     </row>
     <row r="202" ht="15.75" customHeight="1">
-      <c r="A202" s="12"/>
+      <c r="A202" s="13"/>
     </row>
     <row r="203" ht="15.75" customHeight="1">
-      <c r="A203" s="12"/>
+      <c r="A203" s="13"/>
     </row>
     <row r="204" ht="15.75" customHeight="1">
-      <c r="A204" s="12"/>
+      <c r="A204" s="13"/>
     </row>
     <row r="205" ht="15.75" customHeight="1">
-      <c r="A205" s="12"/>
+      <c r="A205" s="13"/>
     </row>
     <row r="206" ht="15.75" customHeight="1">
-      <c r="A206" s="12"/>
+      <c r="A206" s="13"/>
     </row>
     <row r="207" ht="15.75" customHeight="1">
-      <c r="A207" s="12"/>
+      <c r="A207" s="13"/>
     </row>
     <row r="208" ht="15.75" customHeight="1">
-      <c r="A208" s="12"/>
+      <c r="A208" s="13"/>
     </row>
     <row r="209" ht="15.75" customHeight="1">
-      <c r="A209" s="12"/>
+      <c r="A209" s="13"/>
     </row>
     <row r="210" ht="15.75" customHeight="1">
-      <c r="A210" s="12"/>
+      <c r="A210" s="13"/>
     </row>
     <row r="211" ht="15.75" customHeight="1">
-      <c r="A211" s="12"/>
+      <c r="A211" s="13"/>
     </row>
     <row r="212" ht="15.75" customHeight="1">
-      <c r="A212" s="12"/>
+      <c r="A212" s="13"/>
     </row>
     <row r="213" ht="15.75" customHeight="1">
-      <c r="A213" s="12"/>
+      <c r="A213" s="13"/>
     </row>
     <row r="214" ht="15.75" customHeight="1">
-      <c r="A214" s="12"/>
+      <c r="A214" s="13"/>
     </row>
     <row r="215" ht="15.75" customHeight="1">
-      <c r="A215" s="12"/>
+      <c r="A215" s="13"/>
     </row>
     <row r="216" ht="15.75" customHeight="1">
-      <c r="A216" s="12"/>
+      <c r="A216" s="13"/>
     </row>
     <row r="217" ht="15.75" customHeight="1">
-      <c r="A217" s="12"/>
+      <c r="A217" s="13"/>
     </row>
     <row r="218" ht="15.75" customHeight="1">
-      <c r="A218" s="12"/>
+      <c r="A218" s="13"/>
     </row>
     <row r="219" ht="15.75" customHeight="1">
-      <c r="A219" s="12"/>
+      <c r="A219" s="13"/>
     </row>
     <row r="220" ht="15.75" customHeight="1">
-      <c r="A220" s="12"/>
+      <c r="A220" s="13"/>
     </row>
     <row r="221" ht="15.75" customHeight="1">
-      <c r="A221" s="12"/>
+      <c r="A221" s="13"/>
     </row>
     <row r="222" ht="15.75" customHeight="1">
-      <c r="A222" s="12"/>
+      <c r="A222" s="13"/>
     </row>
     <row r="223" ht="15.75" customHeight="1">
-      <c r="A223" s="12"/>
+      <c r="A223" s="13"/>
     </row>
     <row r="224" ht="15.75" customHeight="1">
-      <c r="A224" s="12"/>
+      <c r="A224" s="13"/>
     </row>
     <row r="225" ht="15.75" customHeight="1">
-      <c r="A225" s="12"/>
+      <c r="A225" s="13"/>
     </row>
     <row r="226" ht="15.75" customHeight="1">
-      <c r="A226" s="12"/>
+      <c r="A226" s="13"/>
     </row>
     <row r="227" ht="15.75" customHeight="1">
-      <c r="A227" s="12"/>
+      <c r="A227" s="13"/>
     </row>
     <row r="228" ht="15.75" customHeight="1">
-      <c r="A228" s="12"/>
+      <c r="A228" s="13"/>
     </row>
     <row r="229" ht="15.75" customHeight="1">
-      <c r="A229" s="12"/>
+      <c r="A229" s="13"/>
     </row>
     <row r="230" ht="15.75" customHeight="1">
-      <c r="A230" s="12"/>
+      <c r="A230" s="13"/>
     </row>
     <row r="231" ht="15.75" customHeight="1">
-      <c r="A231" s="12"/>
+      <c r="A231" s="13"/>
     </row>
     <row r="232" ht="15.75" customHeight="1">
-      <c r="A232" s="12"/>
+      <c r="A232" s="13"/>
     </row>
     <row r="233" ht="15.75" customHeight="1">
-      <c r="A233" s="12"/>
+      <c r="A233" s="13"/>
     </row>
     <row r="234" ht="15.75" customHeight="1">
-      <c r="A234" s="12"/>
+      <c r="A234" s="13"/>
     </row>
     <row r="235" ht="15.75" customHeight="1">
-      <c r="A235" s="12"/>
+      <c r="A235" s="13"/>
     </row>
     <row r="236" ht="15.75" customHeight="1">
-      <c r="A236" s="12"/>
+      <c r="A236" s="13"/>
     </row>
     <row r="237" ht="15.75" customHeight="1">
-      <c r="A237" s="12"/>
+      <c r="A237" s="13"/>
     </row>
     <row r="238" ht="15.75" customHeight="1">
-      <c r="A238" s="12"/>
+      <c r="A238" s="13"/>
     </row>
     <row r="239" ht="15.75" customHeight="1">
-      <c r="A239" s="12"/>
+      <c r="A239" s="13"/>
     </row>
     <row r="240" ht="15.75" customHeight="1">
-      <c r="A240" s="12"/>
+      <c r="A240" s="13"/>
     </row>
     <row r="241" ht="15.75" customHeight="1">
-      <c r="A241" s="12"/>
+      <c r="A241" s="13"/>
     </row>
     <row r="242" ht="15.75" customHeight="1">
-      <c r="A242" s="12"/>
+      <c r="A242" s="13"/>
     </row>
     <row r="243" ht="15.75" customHeight="1">
-      <c r="A243" s="12"/>
+      <c r="A243" s="13"/>
     </row>
     <row r="244" ht="15.75" customHeight="1">
-      <c r="A244" s="12"/>
+      <c r="A244" s="13"/>
     </row>
     <row r="245" ht="15.75" customHeight="1">
-      <c r="A245" s="12"/>
+      <c r="A245" s="13"/>
     </row>
     <row r="246" ht="15.75" customHeight="1">
-      <c r="A246" s="12"/>
+      <c r="A246" s="13"/>
     </row>
     <row r="247" ht="15.75" customHeight="1">
-      <c r="A247" s="12"/>
+      <c r="A247" s="13"/>
     </row>
     <row r="248" ht="15.75" customHeight="1">
-      <c r="A248" s="12"/>
+      <c r="A248" s="13"/>
     </row>
     <row r="249" ht="15.75" customHeight="1">
-      <c r="A249" s="12"/>
+      <c r="A249" s="13"/>
     </row>
     <row r="250" ht="15.75" customHeight="1">
-      <c r="A250" s="12"/>
+      <c r="A250" s="13"/>
     </row>
     <row r="251" ht="15.75" customHeight="1">
-      <c r="A251" s="12"/>
+      <c r="A251" s="13"/>
     </row>
     <row r="252" ht="15.75" customHeight="1">
-      <c r="A252" s="12"/>
+      <c r="A252" s="13"/>
     </row>
     <row r="253" ht="15.75" customHeight="1">
-      <c r="A253" s="12"/>
+      <c r="A253" s="13"/>
     </row>
     <row r="254" ht="15.75" customHeight="1">
-      <c r="A254" s="12"/>
+      <c r="A254" s="13"/>
     </row>
     <row r="255" ht="15.75" customHeight="1">
-      <c r="A255" s="12"/>
+      <c r="A255" s="13"/>
     </row>
     <row r="256" ht="15.75" customHeight="1">
-      <c r="A256" s="12"/>
+      <c r="A256" s="13"/>
     </row>
     <row r="257" ht="15.75" customHeight="1">
-      <c r="A257" s="12"/>
+      <c r="A257" s="13"/>
     </row>
     <row r="258" ht="15.75" customHeight="1">
-      <c r="A258" s="12"/>
+      <c r="A258" s="13"/>
     </row>
     <row r="259" ht="15.75" customHeight="1">
-      <c r="A259" s="12"/>
+      <c r="A259" s="13"/>
     </row>
     <row r="260" ht="15.75" customHeight="1">
-      <c r="A260" s="12"/>
+      <c r="A260" s="13"/>
     </row>
     <row r="261" ht="15.75" customHeight="1">
-      <c r="A261" s="12"/>
+      <c r="A261" s="13"/>
     </row>
     <row r="262" ht="15.75" customHeight="1">
-      <c r="A262" s="12"/>
+      <c r="A262" s="13"/>
     </row>
     <row r="263" ht="15.75" customHeight="1">
-      <c r="A263" s="12"/>
+      <c r="A263" s="13"/>
     </row>
     <row r="264" ht="15.75" customHeight="1">
-      <c r="A264" s="12"/>
+      <c r="A264" s="13"/>
     </row>
     <row r="265" ht="15.75" customHeight="1">
-      <c r="A265" s="12"/>
+      <c r="A265" s="13"/>
     </row>
     <row r="266" ht="15.75" customHeight="1">
-      <c r="A266" s="12"/>
+      <c r="A266" s="13"/>
     </row>
     <row r="267" ht="15.75" customHeight="1">
-      <c r="A267" s="12"/>
+      <c r="A267" s="13"/>
     </row>
     <row r="268" ht="15.75" customHeight="1">
-      <c r="A268" s="12"/>
+      <c r="A268" s="13"/>
     </row>
     <row r="269" ht="15.75" customHeight="1">
-      <c r="A269" s="12"/>
+      <c r="A269" s="13"/>
     </row>
     <row r="270" ht="15.75" customHeight="1">
-      <c r="A270" s="12"/>
+      <c r="A270" s="13"/>
     </row>
     <row r="271" ht="15.75" customHeight="1">
-      <c r="A271" s="12"/>
+      <c r="A271" s="13"/>
     </row>
     <row r="272" ht="15.75" customHeight="1">
-      <c r="A272" s="12"/>
+      <c r="A272" s="13"/>
     </row>
     <row r="273" ht="15.75" customHeight="1">
-      <c r="A273" s="12"/>
+      <c r="A273" s="13"/>
     </row>
     <row r="274" ht="15.75" customHeight="1">
-      <c r="A274" s="12"/>
+      <c r="A274" s="13"/>
     </row>
     <row r="275" ht="15.75" customHeight="1">
-      <c r="A275" s="12"/>
+      <c r="A275" s="13"/>
     </row>
     <row r="276" ht="15.75" customHeight="1">
-      <c r="A276" s="12"/>
+      <c r="A276" s="13"/>
     </row>
     <row r="277" ht="15.75" customHeight="1">
-      <c r="A277" s="12"/>
+      <c r="A277" s="13"/>
     </row>
     <row r="278" ht="15.75" customHeight="1">
-      <c r="A278" s="12"/>
+      <c r="A278" s="13"/>
     </row>
     <row r="279" ht="15.75" customHeight="1">
-      <c r="A279" s="12"/>
+      <c r="A279" s="13"/>
     </row>
     <row r="280" ht="15.75" customHeight="1">
-      <c r="A280" s="12"/>
+      <c r="A280" s="13"/>
     </row>
     <row r="281" ht="15.75" customHeight="1">
-      <c r="A281" s="12"/>
+      <c r="A281" s="13"/>
     </row>
     <row r="282" ht="15.75" customHeight="1">
-      <c r="A282" s="12"/>
+      <c r="A282" s="13"/>
     </row>
     <row r="283" ht="15.75" customHeight="1">
-      <c r="A283" s="12"/>
+      <c r="A283" s="13"/>
     </row>
     <row r="284" ht="15.75" customHeight="1">
-      <c r="A284" s="12"/>
+      <c r="A284" s="13"/>
     </row>
     <row r="285" ht="15.75" customHeight="1">
-      <c r="A285" s="12"/>
+      <c r="A285" s="13"/>
     </row>
     <row r="286" ht="15.75" customHeight="1">
-      <c r="A286" s="12"/>
+      <c r="A286" s="13"/>
     </row>
     <row r="287" ht="15.75" customHeight="1">
-      <c r="A287" s="12"/>
+      <c r="A287" s="13"/>
     </row>
     <row r="288" ht="15.75" customHeight="1">
-      <c r="A288" s="12"/>
+      <c r="A288" s="13"/>
     </row>
     <row r="289" ht="15.75" customHeight="1">
-      <c r="A289" s="12"/>
+      <c r="A289" s="13"/>
     </row>
     <row r="290" ht="15.75" customHeight="1">
-      <c r="A290" s="12"/>
+      <c r="A290" s="13"/>
     </row>
     <row r="291" ht="15.75" customHeight="1">
-      <c r="A291" s="12"/>
+      <c r="A291" s="13"/>
     </row>
     <row r="292" ht="15.75" customHeight="1">
-      <c r="A292" s="12"/>
+      <c r="A292" s="13"/>
     </row>
     <row r="293" ht="15.75" customHeight="1">
-      <c r="A293" s="12"/>
+      <c r="A293" s="13"/>
     </row>
     <row r="294" ht="15.75" customHeight="1">
-      <c r="A294" s="12"/>
+      <c r="A294" s="13"/>
     </row>
     <row r="295" ht="15.75" customHeight="1">
-      <c r="A295" s="12"/>
+      <c r="A295" s="13"/>
     </row>
     <row r="296" ht="15.75" customHeight="1">
-      <c r="A296" s="12"/>
+      <c r="A296" s="13"/>
     </row>
     <row r="297" ht="15.75" customHeight="1">
-      <c r="A297" s="12"/>
+      <c r="A297" s="13"/>
     </row>
     <row r="298" ht="15.75" customHeight="1">
-      <c r="A298" s="12"/>
+      <c r="A298" s="13"/>
     </row>
     <row r="299" ht="15.75" customHeight="1">
-      <c r="A299" s="12"/>
+      <c r="A299" s="13"/>
     </row>
     <row r="300" ht="15.75" customHeight="1">
-      <c r="A300" s="12"/>
+      <c r="A300" s="13"/>
     </row>
     <row r="301" ht="15.75" customHeight="1">
-      <c r="A301" s="12"/>
+      <c r="A301" s="13"/>
     </row>
     <row r="302" ht="15.75" customHeight="1">
-      <c r="A302" s="12"/>
+      <c r="A302" s="13"/>
     </row>
     <row r="303" ht="15.75" customHeight="1">
-      <c r="A303" s="12"/>
+      <c r="A303" s="13"/>
     </row>
     <row r="304" ht="15.75" customHeight="1">
-      <c r="A304" s="12"/>
+      <c r="A304" s="13"/>
     </row>
     <row r="305" ht="15.75" customHeight="1">
-      <c r="A305" s="12"/>
+      <c r="A305" s="13"/>
     </row>
     <row r="306" ht="15.75" customHeight="1">
-      <c r="A306" s="12"/>
+      <c r="A306" s="13"/>
     </row>
     <row r="307" ht="15.75" customHeight="1">
-      <c r="A307" s="12"/>
+      <c r="A307" s="13"/>
     </row>
     <row r="308" ht="15.75" customHeight="1">
-      <c r="A308" s="12"/>
+      <c r="A308" s="13"/>
     </row>
     <row r="309" ht="15.75" customHeight="1">
-      <c r="A309" s="12"/>
+      <c r="A309" s="13"/>
     </row>
     <row r="310" ht="15.75" customHeight="1">
-      <c r="A310" s="12"/>
+      <c r="A310" s="13"/>
     </row>
     <row r="311" ht="15.75" customHeight="1">
-      <c r="A311" s="12"/>
+      <c r="A311" s="13"/>
     </row>
     <row r="312" ht="15.75" customHeight="1">
-      <c r="A312" s="12"/>
+      <c r="A312" s="13"/>
     </row>
     <row r="313" ht="15.75" customHeight="1">
-      <c r="A313" s="12"/>
+      <c r="A313" s="13"/>
     </row>
     <row r="314" ht="15.75" customHeight="1">
-      <c r="A314" s="12"/>
+      <c r="A314" s="13"/>
     </row>
     <row r="315" ht="15.75" customHeight="1">
-      <c r="A315" s="12"/>
+      <c r="A315" s="13"/>
     </row>
     <row r="316" ht="15.75" customHeight="1">
-      <c r="A316" s="12"/>
+      <c r="A316" s="13"/>
     </row>
     <row r="317" ht="15.75" customHeight="1">
-      <c r="A317" s="12"/>
+      <c r="A317" s="13"/>
     </row>
     <row r="318" ht="15.75" customHeight="1">
-      <c r="A318" s="12"/>
+      <c r="A318" s="13"/>
     </row>
     <row r="319" ht="15.75" customHeight="1">
-      <c r="A319" s="12"/>
+      <c r="A319" s="13"/>
     </row>
     <row r="320" ht="15.75" customHeight="1">
-      <c r="A320" s="12"/>
+      <c r="A320" s="13"/>
     </row>
     <row r="321" ht="15.75" customHeight="1">
-      <c r="A321" s="12"/>
+      <c r="A321" s="13"/>
     </row>
     <row r="322" ht="15.75" customHeight="1">
-      <c r="A322" s="12"/>
+      <c r="A322" s="13"/>
     </row>
     <row r="323" ht="15.75" customHeight="1">
-      <c r="A323" s="12"/>
+      <c r="A323" s="13"/>
     </row>
     <row r="324" ht="15.75" customHeight="1">
-      <c r="A324" s="12"/>
+      <c r="A324" s="13"/>
     </row>
     <row r="325" ht="15.75" customHeight="1">
-      <c r="A325" s="12"/>
+      <c r="A325" s="13"/>
     </row>
     <row r="326" ht="15.75" customHeight="1">
-      <c r="A326" s="12"/>
+      <c r="A326" s="13"/>
     </row>
     <row r="327" ht="15.75" customHeight="1">
-      <c r="A327" s="12"/>
+      <c r="A327" s="13"/>
     </row>
     <row r="328" ht="15.75" customHeight="1">
-      <c r="A328" s="12"/>
+      <c r="A328" s="13"/>
     </row>
     <row r="329" ht="15.75" customHeight="1">
-      <c r="A329" s="12"/>
+      <c r="A329" s="13"/>
     </row>
     <row r="330" ht="15.75" customHeight="1">
-      <c r="A330" s="12"/>
+      <c r="A330" s="13"/>
     </row>
     <row r="331" ht="15.75" customHeight="1">
-      <c r="A331" s="12"/>
+      <c r="A331" s="13"/>
     </row>
     <row r="332" ht="15.75" customHeight="1">
-      <c r="A332" s="12"/>
+      <c r="A332" s="13"/>
     </row>
     <row r="333" ht="15.75" customHeight="1">
-      <c r="A333" s="12"/>
+      <c r="A333" s="13"/>
     </row>
     <row r="334" ht="15.75" customHeight="1">
-      <c r="A334" s="12"/>
+      <c r="A334" s="13"/>
     </row>
     <row r="335" ht="15.75" customHeight="1">
-      <c r="A335" s="12"/>
+      <c r="A335" s="13"/>
     </row>
     <row r="336" ht="15.75" customHeight="1">
-      <c r="A336" s="12"/>
+      <c r="A336" s="13"/>
     </row>
     <row r="337" ht="15.75" customHeight="1">
-      <c r="A337" s="12"/>
+      <c r="A337" s="13"/>
     </row>
     <row r="338" ht="15.75" customHeight="1">
-      <c r="A338" s="12"/>
+      <c r="A338" s="13"/>
     </row>
     <row r="339" ht="15.75" customHeight="1">
-      <c r="A339" s="12"/>
+      <c r="A339" s="13"/>
     </row>
     <row r="340" ht="15.75" customHeight="1">
-      <c r="A340" s="12"/>
+      <c r="A340" s="13"/>
     </row>
     <row r="341" ht="15.75" customHeight="1">
-      <c r="A341" s="12"/>
+      <c r="A341" s="13"/>
     </row>
     <row r="342" ht="15.75" customHeight="1">
-      <c r="A342" s="12"/>
+      <c r="A342" s="13"/>
     </row>
     <row r="343" ht="15.75" customHeight="1">
-      <c r="A343" s="12"/>
+      <c r="A343" s="13"/>
     </row>
     <row r="344" ht="15.75" customHeight="1">
-      <c r="A344" s="12"/>
+      <c r="A344" s="13"/>
     </row>
     <row r="345" ht="15.75" customHeight="1"/>
     <row r="346" ht="15.75" customHeight="1"/>
@@ -5088,6 +5114,7 @@
     <row r="997" ht="15.75" customHeight="1"/>
     <row r="998" ht="15.75" customHeight="1"/>
     <row r="999" ht="15.75" customHeight="1"/>
+    <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>

</xml_diff>